<commit_message>
ajustes para exportar modelo y documentacion de uso
</commit_message>
<xml_diff>
--- a/output/dashboard_data.xlsx
+++ b/output/dashboard_data.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1_KPIs_Principales" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2_Indicadores_Clave" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3_Lactancia_x_Condicion" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_Complicaciones_Prenatales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5_Hospitalizacion_Detalle" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5b_Hosp_x_Riesgo" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6_Bajo_Peso_Nacer" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="7_Lactancia_General" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="8_Distribucion_Riesgo" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="8b_Riesgo_x_Nutricion" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="9_Resultados_Modelo" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="10_Feature_Importance" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="11a_Edad_Gestacional" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="11b_Sexo" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="11c_Edad_Materna" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_KPIs_Principales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Indicadores_Clave" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Lactancia_x_Condicion" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Complicaciones_Prenatales" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Hospitalizacion_Detalle" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5b_Hosp_x_Riesgo" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Bajo_Peso_Nacer" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Lactancia_General" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Distribucion_Riesgo" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b_Riesgo_x_Nutricion" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_Resultados_Modelo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Feature_Importance" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11a_Edad_Gestacional" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11b_Sexo" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11c_Edad_Materna" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -696,88 +696,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Logistic Regression</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7114</v>
+        <v>0.7727000000000001</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7050999999999999</v>
+        <v>0.7281</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7607</v>
+        <v>0.8329</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7789</v>
+        <v>0.8141</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7675999999999999</v>
+        <v>0.8290999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0105</v>
+        <v>0.0057</v>
       </c>
       <c r="H2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Random Forest</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.767</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.7339</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.8231000000000001</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.8096</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.8234</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Gradient Boosting</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.7768</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.7345</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.8302</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.0049</v>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
@@ -821,10 +761,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.107256517769291</v>
+        <v>0.1773104892630634</v>
       </c>
       <c r="C2" t="n">
-        <v>10.73</v>
+        <v>17.73</v>
       </c>
     </row>
     <row r="3">
@@ -834,10 +774,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0803905263723015</v>
+        <v>0.09839409026891406</v>
       </c>
       <c r="C3" t="n">
-        <v>8.039999999999999</v>
+        <v>9.84</v>
       </c>
     </row>
     <row r="4">
@@ -847,23 +787,23 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.04436027679516453</v>
+        <v>0.08662375609633599</v>
       </c>
       <c r="C4" t="n">
-        <v>4.44</v>
+        <v>8.66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>V196B</t>
+          <t>BMI1</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.02486931849171359</v>
+        <v>0.02641786524256248</v>
       </c>
       <c r="C5" t="n">
-        <v>2.49</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="6">
@@ -873,10 +813,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.02313660343678661</v>
+        <v>0.02572993399161817</v>
       </c>
       <c r="C6" t="n">
-        <v>2.31</v>
+        <v>2.57</v>
       </c>
     </row>
     <row r="7">
@@ -886,322 +826,322 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.02247944055332065</v>
+        <v>0.02064450204978745</v>
       </c>
       <c r="C7" t="n">
-        <v>2.25</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>zscorepeso1</t>
+          <t>CP_TallaMadre</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.02245173948857651</v>
+        <v>0.02064413501295733</v>
       </c>
       <c r="C8" t="n">
-        <v>2.25</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSP_EscolaridadMadre</t>
+          <t>zscorepeso0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.02087145314526716</v>
+        <v>0.01965676051491861</v>
       </c>
       <c r="C9" t="n">
-        <v>2.09</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>zscorepeso0</t>
+          <t>zscoreBMI1</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.02004726850077064</v>
+        <v>0.01941068328471782</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BMI1</t>
+          <t>BMImadre</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0192184974288885</v>
+        <v>0.01861017787745966</v>
       </c>
       <c r="C11" t="n">
-        <v>1.92</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ERN_Peso</t>
+          <t>CP_TallaPadre</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.01890351226627092</v>
+        <v>0.0179094538827317</v>
       </c>
       <c r="C12" t="n">
-        <v>1.89</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ANOCAT</t>
+          <t>zscorepeso1</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.01879611882365115</v>
+        <v>0.01748709263384386</v>
       </c>
       <c r="C13" t="n">
-        <v>1.88</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>primariamadre</t>
+          <t>zscorepesotalla0</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01838386335565115</v>
+        <v>0.01733888629512085</v>
       </c>
       <c r="C14" t="n">
-        <v>1.84</v>
+        <v>1.73</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>zscoreBMI1</t>
+          <t>V196B</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01769492575515798</v>
+        <v>0.01688826462370805</v>
       </c>
       <c r="C15" t="n">
-        <v>1.77</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HD_PesoSalida</t>
+          <t>pesotalla0</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.01764024905518464</v>
+        <v>0.0168497891587378</v>
       </c>
       <c r="C16" t="n">
-        <v>1.76</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>pesotalla0</t>
+          <t>zscorePC0</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0166777771604376</v>
+        <v>0.0147292673585</v>
       </c>
       <c r="C17" t="n">
-        <v>1.67</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>zscorepesotalla0</t>
+          <t>percapindicfinal</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.01651007251061456</v>
+        <v>0.0140917557465222</v>
       </c>
       <c r="C18" t="n">
-        <v>1.65</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>gananciapesonacerpesoentradaPMChosp</t>
+          <t>gananciatallanacertallaentradaPMC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.01592016159827511</v>
+        <v>0.01372514829415903</v>
       </c>
       <c r="C19" t="n">
-        <v>1.59</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>zscorePC0</t>
+          <t>HD_DiasURN</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.01566473288366262</v>
+        <v>0.0133382374186956</v>
       </c>
       <c r="C20" t="n">
-        <v>1.57</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CP_TallaMadre</t>
+          <t>BMIpadre</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.01511117992384588</v>
+        <v>0.01310317713144905</v>
       </c>
       <c r="C21" t="n">
-        <v>1.51</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gananciapesonacerpesoentradaPMC</t>
+          <t>V196C</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.01482887980655799</v>
+        <v>0.01270143687009482</v>
       </c>
       <c r="C22" t="n">
-        <v>1.48</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>zscoretalla1cat</t>
+          <t>ERN_Peso</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.01461363381054145</v>
+        <v>0.01247261802948873</v>
       </c>
       <c r="C23" t="n">
-        <v>1.46</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HD_TotalDiasHospital</t>
+          <t>gananciapesonacerpesoentradaPMChosp</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.01439887876592996</v>
+        <v>0.0121387342063647</v>
       </c>
       <c r="C24" t="n">
-        <v>1.44</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>V196D</t>
+          <t>ANOCAT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.01379029087444618</v>
+        <v>0.01170444765806413</v>
       </c>
       <c r="C25" t="n">
-        <v>1.38</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CP_edadmaterna</t>
+          <t>HD_PesoSalida</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.0136829426387184</v>
+        <v>0.01146487771881079</v>
       </c>
       <c r="C26" t="n">
-        <v>1.37</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HD_DiasURN</t>
+          <t>CP_edadmaterna</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.01367798267363633</v>
+        <v>0.0112850950072551</v>
       </c>
       <c r="C27" t="n">
-        <v>1.37</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BMImadre</t>
+          <t>CP_PesoPadre</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.01331226445778354</v>
+        <v>0.01089306533484459</v>
       </c>
       <c r="C28" t="n">
-        <v>1.33</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>V196C</t>
+          <t>CP_TotalCPN</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.01214677488760686</v>
+        <v>0.01063654730003131</v>
       </c>
       <c r="C29" t="n">
-        <v>1.21</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CP_TallaPadre</t>
+          <t>Sistemadeaseguramiento</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.01165219355203457</v>
+        <v>0.009716637041455964</v>
       </c>
       <c r="C30" t="n">
-        <v>1.17</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>gananciatallanacertallaentradaPMC</t>
+          <t>gananciapesonacerpesoentradaPMC</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.0116253544352688</v>
+        <v>0.009518779096973282</v>
       </c>
       <c r="C31" t="n">
-        <v>1.16</v>
+        <v>0.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>